<commit_message>
Fix hashed-out date columns in the generated sample sheet
Excel never overflows a number/date into an empty neighboring cell the
way it does with text, so with no explicit column width the three date
columns rendered as #### instead of the actual date. Set explicit
per-column widths (generous for the date columns) and regenerated
sample_ar_sheet.xlsx.

Also confirmed (no code change needed): the small-account customers
that stay under Razorpay's real per-link cap were already in the
generator (SMALL_ACCOUNT_CUSTOMERS) — Chi/Upsilon/Phi/Sigma/Rho/Tau all
total ~130k-196k outstanding, comfortably under the 500k cap, so both
"pay this invoice" and "pay everything" always produce a real link for
them instead of the oversized-stub fallback.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_ar_sheet.xlsx
+++ b/sample_ar_sheet.xlsx
@@ -431,6 +431,24 @@
   </sheetPr>
   <dimension ref="A1:P133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -566,10 +584,10 @@
         </is>
       </c>
       <c r="K2" s="2" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>46159</v>
+        <v>46162</v>
       </c>
       <c r="M2" t="n">
         <v>48134.95</v>
@@ -581,7 +599,7 @@
         <v>0</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>46159</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="3">
@@ -636,10 +654,10 @@
         </is>
       </c>
       <c r="K3" s="2" t="n">
-        <v>46173</v>
+        <v>46176</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>46203</v>
+        <v>46206</v>
       </c>
       <c r="M3" t="n">
         <v>231469.93</v>
@@ -651,7 +669,7 @@
         <v>0</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>46203</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="4">
@@ -706,10 +724,10 @@
         </is>
       </c>
       <c r="K4" s="2" t="n">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="M4" t="n">
         <v>415277.68</v>
@@ -774,10 +792,10 @@
         </is>
       </c>
       <c r="K5" s="2" t="n">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="M5" t="n">
         <v>111668.1</v>
@@ -842,10 +860,10 @@
         </is>
       </c>
       <c r="K6" s="2" t="n">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="M6" t="n">
         <v>492453.64</v>
@@ -910,10 +928,10 @@
         </is>
       </c>
       <c r="K7" s="2" t="n">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>46254</v>
+        <v>46257</v>
       </c>
       <c r="M7" t="n">
         <v>544151.6800000001</v>
@@ -978,10 +996,10 @@
         </is>
       </c>
       <c r="K8" s="2" t="n">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>46254</v>
+        <v>46257</v>
       </c>
       <c r="M8" t="n">
         <v>626143.1</v>
@@ -1046,10 +1064,10 @@
         </is>
       </c>
       <c r="K9" s="2" t="n">
-        <v>46049</v>
+        <v>46052</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>46079</v>
+        <v>46082</v>
       </c>
       <c r="M9" t="n">
         <v>228907.58</v>
@@ -1061,7 +1079,7 @@
         <v>0</v>
       </c>
       <c r="P9" s="2" t="n">
-        <v>46079</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="10">
@@ -1116,10 +1134,10 @@
         </is>
       </c>
       <c r="K10" s="2" t="n">
-        <v>46198</v>
+        <v>46201</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>46228</v>
+        <v>46231</v>
       </c>
       <c r="M10" t="n">
         <v>773723.17</v>
@@ -1131,7 +1149,7 @@
         <v>0</v>
       </c>
       <c r="P10" s="2" t="n">
-        <v>46228</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="11">
@@ -1186,10 +1204,10 @@
         </is>
       </c>
       <c r="K11" s="2" t="n">
-        <v>46112</v>
+        <v>46115</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>46142</v>
+        <v>46145</v>
       </c>
       <c r="M11" t="n">
         <v>670778.9399999999</v>
@@ -1201,7 +1219,7 @@
         <v>0</v>
       </c>
       <c r="P11" s="2" t="n">
-        <v>46142</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="12">
@@ -1256,10 +1274,10 @@
         </is>
       </c>
       <c r="K12" s="2" t="n">
-        <v>46232</v>
+        <v>46235</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="M12" t="n">
         <v>224165.23</v>
@@ -1324,10 +1342,10 @@
         </is>
       </c>
       <c r="K13" s="2" t="n">
-        <v>46232</v>
+        <v>46235</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="M13" t="n">
         <v>119544.51</v>
@@ -1392,10 +1410,10 @@
         </is>
       </c>
       <c r="K14" s="2" t="n">
-        <v>46232</v>
+        <v>46235</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="M14" t="n">
         <v>114462.65</v>
@@ -1460,10 +1478,10 @@
         </is>
       </c>
       <c r="K15" s="2" t="n">
-        <v>46082</v>
+        <v>46085</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>46112</v>
+        <v>46115</v>
       </c>
       <c r="M15" t="n">
         <v>771593.65</v>
@@ -1475,7 +1493,7 @@
         <v>0</v>
       </c>
       <c r="P15" s="2" t="n">
-        <v>46112</v>
+        <v>46115</v>
       </c>
     </row>
     <row r="16">
@@ -1530,10 +1548,10 @@
         </is>
       </c>
       <c r="K16" s="2" t="n">
-        <v>46103</v>
+        <v>46106</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>46133</v>
+        <v>46136</v>
       </c>
       <c r="M16" t="n">
         <v>925132.08</v>
@@ -1545,7 +1563,7 @@
         <v>0</v>
       </c>
       <c r="P16" s="2" t="n">
-        <v>46133</v>
+        <v>46136</v>
       </c>
     </row>
     <row r="17">
@@ -1600,10 +1618,10 @@
         </is>
       </c>
       <c r="K17" s="2" t="n">
-        <v>46039</v>
+        <v>46042</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>46069</v>
+        <v>46072</v>
       </c>
       <c r="M17" t="n">
         <v>535637.58</v>
@@ -1615,7 +1633,7 @@
         <v>0</v>
       </c>
       <c r="P17" s="2" t="n">
-        <v>46069</v>
+        <v>46072</v>
       </c>
     </row>
     <row r="18">
@@ -1670,10 +1688,10 @@
         </is>
       </c>
       <c r="K18" s="2" t="n">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="M18" t="n">
         <v>202866.95</v>
@@ -1738,10 +1756,10 @@
         </is>
       </c>
       <c r="K19" s="2" t="n">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="M19" t="n">
         <v>67387.55</v>
@@ -1806,10 +1824,10 @@
         </is>
       </c>
       <c r="K20" s="2" t="n">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="M20" t="n">
         <v>740088.22</v>
@@ -1874,10 +1892,10 @@
         </is>
       </c>
       <c r="K21" s="2" t="n">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="M21" t="n">
         <v>816168.89</v>
@@ -1942,10 +1960,10 @@
         </is>
       </c>
       <c r="K22" s="2" t="n">
-        <v>46232</v>
+        <v>46235</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="M22" t="n">
         <v>376616.76</v>
@@ -2010,10 +2028,10 @@
         </is>
       </c>
       <c r="K23" s="2" t="n">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>46139</v>
+        <v>46142</v>
       </c>
       <c r="M23" t="n">
         <v>175455.04</v>
@@ -2025,7 +2043,7 @@
         <v>0</v>
       </c>
       <c r="P23" s="2" t="n">
-        <v>46145</v>
+        <v>46148</v>
       </c>
     </row>
     <row r="24">
@@ -2080,10 +2098,10 @@
         </is>
       </c>
       <c r="K24" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>46064</v>
+        <v>46067</v>
       </c>
       <c r="M24" t="n">
         <v>644912.04</v>
@@ -2095,7 +2113,7 @@
         <v>0</v>
       </c>
       <c r="P24" s="2" t="n">
-        <v>46066</v>
+        <v>46069</v>
       </c>
     </row>
     <row r="25">
@@ -2150,10 +2168,10 @@
         </is>
       </c>
       <c r="K25" s="2" t="n">
-        <v>46156</v>
+        <v>46159</v>
       </c>
       <c r="L25" s="2" t="n">
-        <v>46186</v>
+        <v>46189</v>
       </c>
       <c r="M25" t="n">
         <v>588446.1800000001</v>
@@ -2165,7 +2183,7 @@
         <v>0</v>
       </c>
       <c r="P25" s="2" t="n">
-        <v>46203</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="26">
@@ -2220,10 +2238,10 @@
         </is>
       </c>
       <c r="K26" s="2" t="n">
-        <v>46201</v>
+        <v>46204</v>
       </c>
       <c r="L26" s="2" t="n">
-        <v>46231</v>
+        <v>46234</v>
       </c>
       <c r="M26" t="n">
         <v>251450.11</v>
@@ -2288,10 +2306,10 @@
         </is>
       </c>
       <c r="K27" s="2" t="n">
-        <v>46217</v>
+        <v>46220</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>46247</v>
+        <v>46250</v>
       </c>
       <c r="M27" t="n">
         <v>375996.28</v>
@@ -2356,10 +2374,10 @@
         </is>
       </c>
       <c r="K28" s="2" t="n">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>46254</v>
+        <v>46257</v>
       </c>
       <c r="M28" t="n">
         <v>658268.1800000001</v>
@@ -2424,10 +2442,10 @@
         </is>
       </c>
       <c r="K29" s="2" t="n">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>46254</v>
+        <v>46257</v>
       </c>
       <c r="M29" t="n">
         <v>236869.47</v>
@@ -2492,10 +2510,10 @@
         </is>
       </c>
       <c r="K30" s="2" t="n">
-        <v>46201</v>
+        <v>46204</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>46231</v>
+        <v>46234</v>
       </c>
       <c r="M30" t="n">
         <v>769667.37</v>
@@ -2560,10 +2578,10 @@
         </is>
       </c>
       <c r="K31" s="2" t="n">
-        <v>46054</v>
+        <v>46057</v>
       </c>
       <c r="L31" s="2" t="n">
-        <v>46084</v>
+        <v>46087</v>
       </c>
       <c r="M31" t="n">
         <v>86224.46000000001</v>
@@ -2575,7 +2593,7 @@
         <v>0</v>
       </c>
       <c r="P31" s="2" t="n">
-        <v>46094</v>
+        <v>46097</v>
       </c>
     </row>
     <row r="32">
@@ -2630,10 +2648,10 @@
         </is>
       </c>
       <c r="K32" s="2" t="n">
-        <v>46072</v>
+        <v>46075</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="M32" t="n">
         <v>221679.55</v>
@@ -2645,7 +2663,7 @@
         <v>0</v>
       </c>
       <c r="P32" s="2" t="n">
-        <v>46114</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="33">
@@ -2700,10 +2718,10 @@
         </is>
       </c>
       <c r="K33" s="2" t="n">
-        <v>46035</v>
+        <v>46038</v>
       </c>
       <c r="L33" s="2" t="n">
-        <v>46065</v>
+        <v>46068</v>
       </c>
       <c r="M33" t="n">
         <v>843331.92</v>
@@ -2715,7 +2733,7 @@
         <v>0</v>
       </c>
       <c r="P33" s="2" t="n">
-        <v>46079</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="34">
@@ -2770,10 +2788,10 @@
         </is>
       </c>
       <c r="K34" s="2" t="n">
-        <v>46217</v>
+        <v>46220</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>46247</v>
+        <v>46250</v>
       </c>
       <c r="M34" t="n">
         <v>270014.15</v>
@@ -2838,10 +2856,10 @@
         </is>
       </c>
       <c r="K35" s="2" t="n">
-        <v>46209</v>
+        <v>46212</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="M35" t="n">
         <v>714114.8100000001</v>
@@ -2906,10 +2924,10 @@
         </is>
       </c>
       <c r="K36" s="2" t="n">
-        <v>46201</v>
+        <v>46204</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>46231</v>
+        <v>46234</v>
       </c>
       <c r="M36" t="n">
         <v>715987.78</v>
@@ -2974,10 +2992,10 @@
         </is>
       </c>
       <c r="K37" s="2" t="n">
-        <v>46164</v>
+        <v>46167</v>
       </c>
       <c r="L37" s="2" t="n">
-        <v>46194</v>
+        <v>46197</v>
       </c>
       <c r="M37" t="n">
         <v>359846.71</v>
@@ -2989,7 +3007,7 @@
         <v>0</v>
       </c>
       <c r="P37" s="2" t="n">
-        <v>46210</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="38">
@@ -3044,10 +3062,10 @@
         </is>
       </c>
       <c r="K38" s="2" t="n">
-        <v>46187</v>
+        <v>46190</v>
       </c>
       <c r="L38" s="2" t="n">
-        <v>46217</v>
+        <v>46220</v>
       </c>
       <c r="M38" t="n">
         <v>481502.15</v>
@@ -3059,7 +3077,7 @@
         <v>0</v>
       </c>
       <c r="P38" s="2" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="39">
@@ -3114,10 +3132,10 @@
         </is>
       </c>
       <c r="K39" s="2" t="n">
-        <v>46159</v>
+        <v>46162</v>
       </c>
       <c r="L39" s="2" t="n">
-        <v>46189</v>
+        <v>46192</v>
       </c>
       <c r="M39" t="n">
         <v>166378.22</v>
@@ -3129,7 +3147,7 @@
         <v>0</v>
       </c>
       <c r="P39" s="2" t="n">
-        <v>46202</v>
+        <v>46205</v>
       </c>
     </row>
     <row r="40">
@@ -3184,10 +3202,10 @@
         </is>
       </c>
       <c r="K40" s="2" t="n">
-        <v>46201</v>
+        <v>46204</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>46231</v>
+        <v>46234</v>
       </c>
       <c r="M40" t="n">
         <v>83763.13</v>
@@ -3252,10 +3270,10 @@
         </is>
       </c>
       <c r="K41" s="2" t="n">
-        <v>46201</v>
+        <v>46204</v>
       </c>
       <c r="L41" s="2" t="n">
-        <v>46231</v>
+        <v>46234</v>
       </c>
       <c r="M41" t="n">
         <v>576196.8</v>
@@ -3320,10 +3338,10 @@
         </is>
       </c>
       <c r="K42" s="2" t="n">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="L42" s="2" t="n">
-        <v>46254</v>
+        <v>46257</v>
       </c>
       <c r="M42" t="n">
         <v>514430.77</v>
@@ -3388,10 +3406,10 @@
         </is>
       </c>
       <c r="K43" s="2" t="n">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="L43" s="2" t="n">
-        <v>46254</v>
+        <v>46257</v>
       </c>
       <c r="M43" t="n">
         <v>654262.15</v>
@@ -3456,10 +3474,10 @@
         </is>
       </c>
       <c r="K44" s="2" t="n">
-        <v>46209</v>
+        <v>46212</v>
       </c>
       <c r="L44" s="2" t="n">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="M44" t="n">
         <v>655582.09</v>
@@ -3524,10 +3542,10 @@
         </is>
       </c>
       <c r="K45" s="2" t="n">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="L45" s="2" t="n">
-        <v>46118</v>
+        <v>46121</v>
       </c>
       <c r="M45" t="n">
         <v>128185.76</v>
@@ -3539,7 +3557,7 @@
         <v>0</v>
       </c>
       <c r="P45" s="2" t="n">
-        <v>46123</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="46">
@@ -3594,10 +3612,10 @@
         </is>
       </c>
       <c r="K46" s="2" t="n">
-        <v>46132</v>
+        <v>46135</v>
       </c>
       <c r="L46" s="2" t="n">
-        <v>46162</v>
+        <v>46165</v>
       </c>
       <c r="M46" t="n">
         <v>444694.43</v>
@@ -3609,7 +3627,7 @@
         <v>0</v>
       </c>
       <c r="P46" s="2" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="47">
@@ -3664,10 +3682,10 @@
         </is>
       </c>
       <c r="K47" s="2" t="n">
-        <v>46070</v>
+        <v>46073</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>46100</v>
+        <v>46103</v>
       </c>
       <c r="M47" t="n">
         <v>729815.03</v>
@@ -3679,7 +3697,7 @@
         <v>0</v>
       </c>
       <c r="P47" s="2" t="n">
-        <v>46103</v>
+        <v>46106</v>
       </c>
     </row>
     <row r="48">
@@ -3734,10 +3752,10 @@
         </is>
       </c>
       <c r="K48" s="2" t="n">
-        <v>46217</v>
+        <v>46220</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>46247</v>
+        <v>46250</v>
       </c>
       <c r="M48" t="n">
         <v>301061.43</v>
@@ -3802,10 +3820,10 @@
         </is>
       </c>
       <c r="K49" s="2" t="n">
-        <v>46217</v>
+        <v>46220</v>
       </c>
       <c r="L49" s="2" t="n">
-        <v>46247</v>
+        <v>46250</v>
       </c>
       <c r="M49" t="n">
         <v>166376.32</v>
@@ -3870,10 +3888,10 @@
         </is>
       </c>
       <c r="K50" s="2" t="n">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="L50" s="2" t="n">
-        <v>46254</v>
+        <v>46257</v>
       </c>
       <c r="M50" t="n">
         <v>523925.6</v>
@@ -3938,10 +3956,10 @@
         </is>
       </c>
       <c r="K51" s="2" t="n">
-        <v>46201</v>
+        <v>46204</v>
       </c>
       <c r="L51" s="2" t="n">
-        <v>46231</v>
+        <v>46234</v>
       </c>
       <c r="M51" t="n">
         <v>579023.74</v>
@@ -4006,10 +4024,10 @@
         </is>
       </c>
       <c r="K52" s="2" t="n">
-        <v>46209</v>
+        <v>46212</v>
       </c>
       <c r="L52" s="2" t="n">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="M52" t="n">
         <v>43015.99</v>
@@ -4074,10 +4092,10 @@
         </is>
       </c>
       <c r="K53" s="2" t="n">
-        <v>46138</v>
+        <v>46141</v>
       </c>
       <c r="L53" s="2" t="n">
-        <v>46168</v>
+        <v>46171</v>
       </c>
       <c r="M53" t="n">
         <v>246493.39</v>
@@ -4089,7 +4107,7 @@
         <v>0</v>
       </c>
       <c r="P53" s="2" t="n">
-        <v>46186</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="54">
@@ -4144,10 +4162,10 @@
         </is>
       </c>
       <c r="K54" s="2" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="L54" s="2" t="n">
-        <v>46208</v>
+        <v>46211</v>
       </c>
       <c r="M54" t="n">
         <v>900928.24</v>
@@ -4159,7 +4177,7 @@
         <v>0</v>
       </c>
       <c r="P54" s="2" t="n">
-        <v>46223</v>
+        <v>46226</v>
       </c>
     </row>
     <row r="55">
@@ -4214,10 +4232,10 @@
         </is>
       </c>
       <c r="K55" s="2" t="n">
-        <v>46063</v>
+        <v>46066</v>
       </c>
       <c r="L55" s="2" t="n">
-        <v>46093</v>
+        <v>46096</v>
       </c>
       <c r="M55" t="n">
         <v>779821.51</v>
@@ -4229,7 +4247,7 @@
         <v>0</v>
       </c>
       <c r="P55" s="2" t="n">
-        <v>46097</v>
+        <v>46100</v>
       </c>
     </row>
     <row r="56">
@@ -4284,10 +4302,10 @@
         </is>
       </c>
       <c r="K56" s="2" t="n">
-        <v>46217</v>
+        <v>46220</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>46247</v>
+        <v>46250</v>
       </c>
       <c r="M56" t="n">
         <v>635269.51</v>
@@ -4352,10 +4370,10 @@
         </is>
       </c>
       <c r="K57" s="2" t="n">
-        <v>46201</v>
+        <v>46204</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>46231</v>
+        <v>46234</v>
       </c>
       <c r="M57" t="n">
         <v>270177.38</v>
@@ -4420,10 +4438,10 @@
         </is>
       </c>
       <c r="K58" s="2" t="n">
-        <v>46217</v>
+        <v>46220</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>46247</v>
+        <v>46250</v>
       </c>
       <c r="M58" t="n">
         <v>917035.6899999999</v>
@@ -4488,10 +4506,10 @@
         </is>
       </c>
       <c r="K59" s="2" t="n">
-        <v>46033</v>
+        <v>46036</v>
       </c>
       <c r="L59" s="2" t="n">
-        <v>46063</v>
+        <v>46066</v>
       </c>
       <c r="M59" t="n">
         <v>394067.88</v>
@@ -4503,7 +4521,7 @@
         <v>0</v>
       </c>
       <c r="P59" s="2" t="n">
-        <v>46074</v>
+        <v>46077</v>
       </c>
     </row>
     <row r="60">
@@ -4558,10 +4576,10 @@
         </is>
       </c>
       <c r="K60" s="2" t="n">
-        <v>46067</v>
+        <v>46070</v>
       </c>
       <c r="L60" s="2" t="n">
-        <v>46097</v>
+        <v>46100</v>
       </c>
       <c r="M60" t="n">
         <v>430242.58</v>
@@ -4573,7 +4591,7 @@
         <v>0</v>
       </c>
       <c r="P60" s="2" t="n">
-        <v>46111</v>
+        <v>46114</v>
       </c>
     </row>
     <row r="61">
@@ -4628,10 +4646,10 @@
         </is>
       </c>
       <c r="K61" s="2" t="n">
-        <v>46142</v>
+        <v>46145</v>
       </c>
       <c r="L61" s="2" t="n">
-        <v>46172</v>
+        <v>46175</v>
       </c>
       <c r="M61" t="n">
         <v>136928.88</v>
@@ -4643,7 +4661,7 @@
         <v>0</v>
       </c>
       <c r="P61" s="2" t="n">
-        <v>46174</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="62">
@@ -4698,10 +4716,10 @@
         </is>
       </c>
       <c r="K62" s="2" t="n">
-        <v>46217</v>
+        <v>46220</v>
       </c>
       <c r="L62" s="2" t="n">
-        <v>46247</v>
+        <v>46250</v>
       </c>
       <c r="M62" t="n">
         <v>44456.69</v>
@@ -4766,10 +4784,10 @@
         </is>
       </c>
       <c r="K63" s="2" t="n">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="L63" s="2" t="n">
-        <v>46254</v>
+        <v>46257</v>
       </c>
       <c r="M63" t="n">
         <v>569307.11</v>
@@ -4834,10 +4852,10 @@
         </is>
       </c>
       <c r="K64" s="2" t="n">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="L64" s="2" t="n">
-        <v>46254</v>
+        <v>46257</v>
       </c>
       <c r="M64" t="n">
         <v>90668.60000000001</v>
@@ -4902,10 +4920,10 @@
         </is>
       </c>
       <c r="K65" s="2" t="n">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="L65" s="2" t="n">
-        <v>46254</v>
+        <v>46257</v>
       </c>
       <c r="M65" t="n">
         <v>236771.15</v>
@@ -4970,10 +4988,10 @@
         </is>
       </c>
       <c r="K66" s="2" t="n">
-        <v>46139</v>
+        <v>46142</v>
       </c>
       <c r="L66" s="2" t="n">
-        <v>46169</v>
+        <v>46172</v>
       </c>
       <c r="M66" t="n">
         <v>90543.05</v>
@@ -4985,7 +5003,7 @@
         <v>0</v>
       </c>
       <c r="P66" s="2" t="n">
-        <v>46201</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="67">
@@ -5040,10 +5058,10 @@
         </is>
       </c>
       <c r="K67" s="2" t="n">
-        <v>46145</v>
+        <v>46148</v>
       </c>
       <c r="L67" s="2" t="n">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="M67" t="n">
         <v>643804.4399999999</v>
@@ -5055,7 +5073,7 @@
         <v>0</v>
       </c>
       <c r="P67" s="2" t="n">
-        <v>46224</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="68">
@@ -5110,10 +5128,10 @@
         </is>
       </c>
       <c r="K68" s="2" t="n">
-        <v>46053</v>
+        <v>46056</v>
       </c>
       <c r="L68" s="2" t="n">
-        <v>46083</v>
+        <v>46086</v>
       </c>
       <c r="M68" t="n">
         <v>147388.46</v>
@@ -5125,7 +5143,7 @@
         <v>0</v>
       </c>
       <c r="P68" s="2" t="n">
-        <v>46134</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="69">
@@ -5180,10 +5198,10 @@
         </is>
       </c>
       <c r="K69" s="2" t="n">
-        <v>46149</v>
+        <v>46152</v>
       </c>
       <c r="L69" s="2" t="n">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="M69" t="n">
         <v>249772.45</v>
@@ -5248,10 +5266,10 @@
         </is>
       </c>
       <c r="K70" s="2" t="n">
-        <v>46184</v>
+        <v>46187</v>
       </c>
       <c r="L70" s="2" t="n">
-        <v>46214</v>
+        <v>46217</v>
       </c>
       <c r="M70" t="n">
         <v>771934.72</v>
@@ -5316,10 +5334,10 @@
         </is>
       </c>
       <c r="K71" s="2" t="n">
-        <v>46149</v>
+        <v>46152</v>
       </c>
       <c r="L71" s="2" t="n">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="M71" t="n">
         <v>112251.36</v>
@@ -5384,10 +5402,10 @@
         </is>
       </c>
       <c r="K72" s="2" t="n">
-        <v>46149</v>
+        <v>46152</v>
       </c>
       <c r="L72" s="2" t="n">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="M72" t="n">
         <v>352725.25</v>
@@ -5452,10 +5470,10 @@
         </is>
       </c>
       <c r="K73" s="2" t="n">
-        <v>46186</v>
+        <v>46189</v>
       </c>
       <c r="L73" s="2" t="n">
-        <v>46216</v>
+        <v>46219</v>
       </c>
       <c r="M73" t="n">
         <v>824048.99</v>
@@ -5467,7 +5485,7 @@
         <v>0</v>
       </c>
       <c r="P73" s="2" t="n">
-        <v>46274</v>
+        <v>46277</v>
       </c>
     </row>
     <row r="74">
@@ -5522,10 +5540,10 @@
         </is>
       </c>
       <c r="K74" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="L74" s="2" t="n">
-        <v>46064</v>
+        <v>46067</v>
       </c>
       <c r="M74" t="n">
         <v>629446.33</v>
@@ -5537,7 +5555,7 @@
         <v>0</v>
       </c>
       <c r="P74" s="2" t="n">
-        <v>46085</v>
+        <v>46088</v>
       </c>
     </row>
     <row r="75">
@@ -5592,10 +5610,10 @@
         </is>
       </c>
       <c r="K75" s="2" t="n">
-        <v>46113</v>
+        <v>46116</v>
       </c>
       <c r="L75" s="2" t="n">
-        <v>46143</v>
+        <v>46146</v>
       </c>
       <c r="M75" t="n">
         <v>81066.72</v>
@@ -5607,7 +5625,7 @@
         <v>0</v>
       </c>
       <c r="P75" s="2" t="n">
-        <v>46164</v>
+        <v>46167</v>
       </c>
     </row>
     <row r="76">
@@ -5662,10 +5680,10 @@
         </is>
       </c>
       <c r="K76" s="2" t="n">
-        <v>46149</v>
+        <v>46152</v>
       </c>
       <c r="L76" s="2" t="n">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="M76" t="n">
         <v>202220.82</v>
@@ -5730,10 +5748,10 @@
         </is>
       </c>
       <c r="K77" s="2" t="n">
-        <v>46184</v>
+        <v>46187</v>
       </c>
       <c r="L77" s="2" t="n">
-        <v>46214</v>
+        <v>46217</v>
       </c>
       <c r="M77" t="n">
         <v>154668.62</v>
@@ -5798,10 +5816,10 @@
         </is>
       </c>
       <c r="K78" s="2" t="n">
-        <v>46184</v>
+        <v>46187</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>46214</v>
+        <v>46217</v>
       </c>
       <c r="M78" t="n">
         <v>282654.26</v>
@@ -5866,10 +5884,10 @@
         </is>
       </c>
       <c r="K79" s="2" t="n">
-        <v>46059</v>
+        <v>46062</v>
       </c>
       <c r="L79" s="2" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="M79" t="n">
         <v>434895.94</v>
@@ -5881,7 +5899,7 @@
         <v>0</v>
       </c>
       <c r="P79" s="2" t="n">
-        <v>46110</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="80">
@@ -5936,10 +5954,10 @@
         </is>
       </c>
       <c r="K80" s="2" t="n">
-        <v>46061</v>
+        <v>46064</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="M80" t="n">
         <v>71794.2</v>
@@ -5951,7 +5969,7 @@
         <v>0</v>
       </c>
       <c r="P80" s="2" t="n">
-        <v>46106</v>
+        <v>46109</v>
       </c>
     </row>
     <row r="81">
@@ -6006,10 +6024,10 @@
         </is>
       </c>
       <c r="K81" s="2" t="n">
-        <v>46184</v>
+        <v>46187</v>
       </c>
       <c r="L81" s="2" t="n">
-        <v>46214</v>
+        <v>46217</v>
       </c>
       <c r="M81" t="n">
         <v>881889.46</v>
@@ -6074,10 +6092,10 @@
         </is>
       </c>
       <c r="K82" s="2" t="n">
-        <v>46149</v>
+        <v>46152</v>
       </c>
       <c r="L82" s="2" t="n">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="M82" t="n">
         <v>178837.78</v>
@@ -6142,10 +6160,10 @@
         </is>
       </c>
       <c r="K83" s="2" t="n">
-        <v>46149</v>
+        <v>46152</v>
       </c>
       <c r="L83" s="2" t="n">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="M83" t="n">
         <v>470256.54</v>
@@ -6210,10 +6228,10 @@
         </is>
       </c>
       <c r="K84" s="2" t="n">
-        <v>46199</v>
+        <v>46202</v>
       </c>
       <c r="L84" s="2" t="n">
-        <v>46229</v>
+        <v>46232</v>
       </c>
       <c r="M84" t="n">
         <v>177289.34</v>
@@ -6225,7 +6243,7 @@
         <v>0</v>
       </c>
       <c r="P84" s="2" t="n">
-        <v>46268</v>
+        <v>46271</v>
       </c>
     </row>
     <row r="85">
@@ -6280,10 +6298,10 @@
         </is>
       </c>
       <c r="K85" s="2" t="n">
-        <v>46083</v>
+        <v>46086</v>
       </c>
       <c r="L85" s="2" t="n">
-        <v>46113</v>
+        <v>46116</v>
       </c>
       <c r="M85" t="n">
         <v>270312.83</v>
@@ -6295,7 +6313,7 @@
         <v>0</v>
       </c>
       <c r="P85" s="2" t="n">
-        <v>46146</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="86">
@@ -6350,10 +6368,10 @@
         </is>
       </c>
       <c r="K86" s="2" t="n">
-        <v>46149</v>
+        <v>46152</v>
       </c>
       <c r="L86" s="2" t="n">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="M86" t="n">
         <v>669347.14</v>
@@ -6418,10 +6436,10 @@
         </is>
       </c>
       <c r="K87" s="2" t="n">
-        <v>46164</v>
+        <v>46167</v>
       </c>
       <c r="L87" s="2" t="n">
-        <v>46194</v>
+        <v>46197</v>
       </c>
       <c r="M87" t="n">
         <v>168187.06</v>
@@ -6486,10 +6504,10 @@
         </is>
       </c>
       <c r="K88" s="2" t="n">
-        <v>46194</v>
+        <v>46197</v>
       </c>
       <c r="L88" s="2" t="n">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="M88" t="n">
         <v>226373.33</v>
@@ -6554,10 +6572,10 @@
         </is>
       </c>
       <c r="K89" s="2" t="n">
-        <v>46194</v>
+        <v>46197</v>
       </c>
       <c r="L89" s="2" t="n">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="M89" t="n">
         <v>560741.77</v>
@@ -6622,10 +6640,10 @@
         </is>
       </c>
       <c r="K90" s="2" t="n">
-        <v>46050</v>
+        <v>46053</v>
       </c>
       <c r="L90" s="2" t="n">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="M90" t="n">
         <v>77877.88</v>
@@ -6637,7 +6655,7 @@
         <v>0</v>
       </c>
       <c r="P90" s="2" t="n">
-        <v>46181</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="91">
@@ -6692,10 +6710,10 @@
         </is>
       </c>
       <c r="K91" s="2" t="n">
-        <v>46064</v>
+        <v>46067</v>
       </c>
       <c r="L91" s="2" t="n">
-        <v>46094</v>
+        <v>46097</v>
       </c>
       <c r="M91" t="n">
         <v>490136.6</v>
@@ -6707,7 +6725,7 @@
         <v>0</v>
       </c>
       <c r="P91" s="2" t="n">
-        <v>46154</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="92">
@@ -6762,10 +6780,10 @@
         </is>
       </c>
       <c r="K92" s="2" t="n">
-        <v>46069</v>
+        <v>46072</v>
       </c>
       <c r="L92" s="2" t="n">
-        <v>46099</v>
+        <v>46102</v>
       </c>
       <c r="M92" t="n">
         <v>77613.61</v>
@@ -6777,7 +6795,7 @@
         <v>0</v>
       </c>
       <c r="P92" s="2" t="n">
-        <v>46149</v>
+        <v>46152</v>
       </c>
     </row>
     <row r="93">
@@ -6832,10 +6850,10 @@
         </is>
       </c>
       <c r="K93" s="2" t="n">
-        <v>46159</v>
+        <v>46162</v>
       </c>
       <c r="L93" s="2" t="n">
-        <v>46189</v>
+        <v>46192</v>
       </c>
       <c r="M93" t="n">
         <v>88382.23</v>
@@ -6900,10 +6918,10 @@
         </is>
       </c>
       <c r="K94" s="2" t="n">
-        <v>46134</v>
+        <v>46137</v>
       </c>
       <c r="L94" s="2" t="n">
-        <v>46164</v>
+        <v>46167</v>
       </c>
       <c r="M94" t="n">
         <v>649571.61</v>
@@ -6968,10 +6986,10 @@
         </is>
       </c>
       <c r="K95" s="2" t="n">
-        <v>46134</v>
+        <v>46137</v>
       </c>
       <c r="L95" s="2" t="n">
-        <v>46164</v>
+        <v>46167</v>
       </c>
       <c r="M95" t="n">
         <v>398492.38</v>
@@ -7036,10 +7054,10 @@
         </is>
       </c>
       <c r="K96" s="2" t="n">
-        <v>46092</v>
+        <v>46095</v>
       </c>
       <c r="L96" s="2" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="M96" t="n">
         <v>597927.9</v>
@@ -7051,7 +7069,7 @@
         <v>0</v>
       </c>
       <c r="P96" s="2" t="n">
-        <v>46236</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="97">
@@ -7106,10 +7124,10 @@
         </is>
       </c>
       <c r="K97" s="2" t="n">
-        <v>46119</v>
+        <v>46122</v>
       </c>
       <c r="L97" s="2" t="n">
-        <v>46149</v>
+        <v>46152</v>
       </c>
       <c r="M97" t="n">
         <v>547834.9</v>
@@ -7121,7 +7139,7 @@
         <v>0</v>
       </c>
       <c r="P97" s="2" t="n">
-        <v>46222</v>
+        <v>46225</v>
       </c>
     </row>
     <row r="98">
@@ -7176,10 +7194,10 @@
         </is>
       </c>
       <c r="K98" s="2" t="n">
-        <v>46119</v>
+        <v>46122</v>
       </c>
       <c r="L98" s="2" t="n">
-        <v>46149</v>
+        <v>46152</v>
       </c>
       <c r="M98" t="n">
         <v>644496.53</v>
@@ -7244,10 +7262,10 @@
         </is>
       </c>
       <c r="K99" s="2" t="n">
-        <v>46099</v>
+        <v>46102</v>
       </c>
       <c r="L99" s="2" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="M99" t="n">
         <v>245784.51</v>
@@ -7312,10 +7330,10 @@
         </is>
       </c>
       <c r="K100" s="2" t="n">
-        <v>46119</v>
+        <v>46122</v>
       </c>
       <c r="L100" s="2" t="n">
-        <v>46149</v>
+        <v>46152</v>
       </c>
       <c r="M100" t="n">
         <v>146062.41</v>
@@ -7380,10 +7398,10 @@
         </is>
       </c>
       <c r="K101" s="2" t="n">
-        <v>46181</v>
+        <v>46184</v>
       </c>
       <c r="L101" s="2" t="n">
-        <v>46211</v>
+        <v>46214</v>
       </c>
       <c r="M101" t="n">
         <v>317463.91</v>
@@ -7395,7 +7413,7 @@
         <v>0</v>
       </c>
       <c r="P101" s="2" t="n">
-        <v>46252</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="102">
@@ -7450,10 +7468,10 @@
         </is>
       </c>
       <c r="K102" s="2" t="n">
-        <v>46055</v>
+        <v>46058</v>
       </c>
       <c r="L102" s="2" t="n">
-        <v>46085</v>
+        <v>46088</v>
       </c>
       <c r="M102" t="n">
         <v>448914.11</v>
@@ -7465,7 +7483,7 @@
         <v>0</v>
       </c>
       <c r="P102" s="2" t="n">
-        <v>46137</v>
+        <v>46140</v>
       </c>
     </row>
     <row r="103">
@@ -7520,10 +7538,10 @@
         </is>
       </c>
       <c r="K103" s="2" t="n">
-        <v>46145</v>
+        <v>46148</v>
       </c>
       <c r="L103" s="2" t="n">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="M103" t="n">
         <v>92766.17</v>
@@ -7535,7 +7553,7 @@
         <v>0</v>
       </c>
       <c r="P103" s="2" t="n">
-        <v>46279</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="104">
@@ -7590,10 +7608,10 @@
         </is>
       </c>
       <c r="K104" s="2" t="n">
-        <v>46119</v>
+        <v>46122</v>
       </c>
       <c r="L104" s="2" t="n">
-        <v>46149</v>
+        <v>46152</v>
       </c>
       <c r="M104" t="n">
         <v>147522.33</v>
@@ -7658,10 +7676,10 @@
         </is>
       </c>
       <c r="K105" s="2" t="n">
-        <v>46134</v>
+        <v>46137</v>
       </c>
       <c r="L105" s="2" t="n">
-        <v>46164</v>
+        <v>46167</v>
       </c>
       <c r="M105" t="n">
         <v>839799.36</v>
@@ -7726,10 +7744,10 @@
         </is>
       </c>
       <c r="K106" s="2" t="n">
-        <v>46134</v>
+        <v>46137</v>
       </c>
       <c r="L106" s="2" t="n">
-        <v>46164</v>
+        <v>46167</v>
       </c>
       <c r="M106" t="n">
         <v>366812.56</v>
@@ -7794,10 +7812,10 @@
         </is>
       </c>
       <c r="K107" s="2" t="n">
-        <v>46119</v>
+        <v>46122</v>
       </c>
       <c r="L107" s="2" t="n">
-        <v>46149</v>
+        <v>46152</v>
       </c>
       <c r="M107" t="n">
         <v>430320.73</v>
@@ -7862,10 +7880,10 @@
         </is>
       </c>
       <c r="K108" s="2" t="n">
-        <v>46058</v>
+        <v>46061</v>
       </c>
       <c r="L108" s="2" t="n">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="M108" t="n">
         <v>642773.46</v>
@@ -7877,7 +7895,7 @@
         <v>0</v>
       </c>
       <c r="P108" s="2" t="n">
-        <v>46088</v>
+        <v>46091</v>
       </c>
     </row>
     <row r="109">
@@ -7932,10 +7950,10 @@
         </is>
       </c>
       <c r="K109" s="2" t="n">
-        <v>46173</v>
+        <v>46176</v>
       </c>
       <c r="L109" s="2" t="n">
-        <v>46203</v>
+        <v>46206</v>
       </c>
       <c r="M109" t="n">
         <v>886874.34</v>
@@ -7947,7 +7965,7 @@
         <v>0</v>
       </c>
       <c r="P109" s="2" t="n">
-        <v>46203</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="110">
@@ -8002,10 +8020,10 @@
         </is>
       </c>
       <c r="K110" s="2" t="n">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="L110" s="2" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="M110" t="n">
         <v>39428.58</v>
@@ -8070,10 +8088,10 @@
         </is>
       </c>
       <c r="K111" s="2" t="n">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="L111" s="2" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="M111" t="n">
         <v>117802.09</v>
@@ -8138,10 +8156,10 @@
         </is>
       </c>
       <c r="K112" s="2" t="n">
-        <v>46146</v>
+        <v>46149</v>
       </c>
       <c r="L112" s="2" t="n">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="M112" t="n">
         <v>285624.55</v>
@@ -8153,7 +8171,7 @@
         <v>0</v>
       </c>
       <c r="P112" s="2" t="n">
-        <v>46186</v>
+        <v>46189</v>
       </c>
     </row>
     <row r="113">
@@ -8208,10 +8226,10 @@
         </is>
       </c>
       <c r="K113" s="2" t="n">
-        <v>46037</v>
+        <v>46040</v>
       </c>
       <c r="L113" s="2" t="n">
-        <v>46067</v>
+        <v>46070</v>
       </c>
       <c r="M113" t="n">
         <v>213327.51</v>
@@ -8223,7 +8241,7 @@
         <v>0</v>
       </c>
       <c r="P113" s="2" t="n">
-        <v>46075</v>
+        <v>46078</v>
       </c>
     </row>
     <row r="114">
@@ -8278,10 +8296,10 @@
         </is>
       </c>
       <c r="K114" s="2" t="n">
-        <v>46135</v>
+        <v>46138</v>
       </c>
       <c r="L114" s="2" t="n">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="M114" t="n">
         <v>492503.38</v>
@@ -8293,7 +8311,7 @@
         <v>0</v>
       </c>
       <c r="P114" s="2" t="n">
-        <v>46166</v>
+        <v>46169</v>
       </c>
     </row>
     <row r="115">
@@ -8348,10 +8366,10 @@
         </is>
       </c>
       <c r="K115" s="2" t="n">
-        <v>46209</v>
+        <v>46212</v>
       </c>
       <c r="L115" s="2" t="n">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="M115" t="n">
         <v>104285.56</v>
@@ -8416,10 +8434,10 @@
         </is>
       </c>
       <c r="K116" s="2" t="n">
-        <v>46209</v>
+        <v>46212</v>
       </c>
       <c r="L116" s="2" t="n">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="M116" t="n">
         <v>30510.85</v>
@@ -8484,10 +8502,10 @@
         </is>
       </c>
       <c r="K117" s="2" t="n">
-        <v>46132</v>
+        <v>46135</v>
       </c>
       <c r="L117" s="2" t="n">
-        <v>46162</v>
+        <v>46165</v>
       </c>
       <c r="M117" t="n">
         <v>614329.87</v>
@@ -8499,7 +8517,7 @@
         <v>0</v>
       </c>
       <c r="P117" s="2" t="n">
-        <v>46167</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="118">
@@ -8554,10 +8572,10 @@
         </is>
       </c>
       <c r="K118" s="2" t="n">
-        <v>46058</v>
+        <v>46061</v>
       </c>
       <c r="L118" s="2" t="n">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="M118" t="n">
         <v>710638.59</v>
@@ -8569,7 +8587,7 @@
         <v>0</v>
       </c>
       <c r="P118" s="2" t="n">
-        <v>46101</v>
+        <v>46104</v>
       </c>
     </row>
     <row r="119">
@@ -8624,10 +8642,10 @@
         </is>
       </c>
       <c r="K119" s="2" t="n">
-        <v>46217</v>
+        <v>46220</v>
       </c>
       <c r="L119" s="2" t="n">
-        <v>46247</v>
+        <v>46250</v>
       </c>
       <c r="M119" t="n">
         <v>38984.24</v>
@@ -8692,10 +8710,10 @@
         </is>
       </c>
       <c r="K120" s="2" t="n">
-        <v>46209</v>
+        <v>46212</v>
       </c>
       <c r="L120" s="2" t="n">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="M120" t="n">
         <v>93198.78999999999</v>
@@ -8760,10 +8778,10 @@
         </is>
       </c>
       <c r="K121" s="2" t="n">
-        <v>46189</v>
+        <v>46192</v>
       </c>
       <c r="L121" s="2" t="n">
-        <v>46219</v>
+        <v>46222</v>
       </c>
       <c r="M121" t="n">
         <v>422552.71</v>
@@ -8775,7 +8793,7 @@
         <v>0</v>
       </c>
       <c r="P121" s="2" t="n">
-        <v>46253</v>
+        <v>46256</v>
       </c>
     </row>
     <row r="122">
@@ -8830,10 +8848,10 @@
         </is>
       </c>
       <c r="K122" s="2" t="n">
-        <v>46189</v>
+        <v>46192</v>
       </c>
       <c r="L122" s="2" t="n">
-        <v>46219</v>
+        <v>46222</v>
       </c>
       <c r="M122" t="n">
         <v>362302.65</v>
@@ -8845,7 +8863,7 @@
         <v>0</v>
       </c>
       <c r="P122" s="2" t="n">
-        <v>46256</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="123">
@@ -8900,10 +8918,10 @@
         </is>
       </c>
       <c r="K123" s="2" t="n">
-        <v>46194</v>
+        <v>46197</v>
       </c>
       <c r="L123" s="2" t="n">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="M123" t="n">
         <v>110258.34</v>
@@ -8968,10 +8986,10 @@
         </is>
       </c>
       <c r="K124" s="2" t="n">
-        <v>46149</v>
+        <v>46152</v>
       </c>
       <c r="L124" s="2" t="n">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="M124" t="n">
         <v>69209.83</v>
@@ -9036,10 +9054,10 @@
         </is>
       </c>
       <c r="K125" s="2" t="n">
-        <v>46139</v>
+        <v>46142</v>
       </c>
       <c r="L125" s="2" t="n">
-        <v>46169</v>
+        <v>46172</v>
       </c>
       <c r="M125" t="n">
         <v>881331.54</v>
@@ -9051,7 +9069,7 @@
         <v>0</v>
       </c>
       <c r="P125" s="2" t="n">
-        <v>46169</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="126">
@@ -9106,10 +9124,10 @@
         </is>
       </c>
       <c r="K126" s="2" t="n">
-        <v>46154</v>
+        <v>46157</v>
       </c>
       <c r="L126" s="2" t="n">
-        <v>46184</v>
+        <v>46187</v>
       </c>
       <c r="M126" t="n">
         <v>927990.58</v>
@@ -9121,7 +9139,7 @@
         <v>0</v>
       </c>
       <c r="P126" s="2" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="127">
@@ -9176,10 +9194,10 @@
         </is>
       </c>
       <c r="K127" s="2" t="n">
-        <v>46232</v>
+        <v>46235</v>
       </c>
       <c r="L127" s="2" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="M127" t="n">
         <v>47420.08</v>
@@ -9244,10 +9262,10 @@
         </is>
       </c>
       <c r="K128" s="2" t="n">
-        <v>46232</v>
+        <v>46235</v>
       </c>
       <c r="L128" s="2" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="M128" t="n">
         <v>122798.31</v>
@@ -9312,10 +9330,10 @@
         </is>
       </c>
       <c r="K129" s="2" t="n">
-        <v>46172</v>
+        <v>46175</v>
       </c>
       <c r="L129" s="2" t="n">
-        <v>46202</v>
+        <v>46205</v>
       </c>
       <c r="M129" t="n">
         <v>271795.28</v>
@@ -9327,7 +9345,7 @@
         <v>0</v>
       </c>
       <c r="P129" s="2" t="n">
-        <v>46290</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="130">
@@ -9382,10 +9400,10 @@
         </is>
       </c>
       <c r="K130" s="2" t="n">
-        <v>46079</v>
+        <v>46082</v>
       </c>
       <c r="L130" s="2" t="n">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="M130" t="n">
         <v>831754.27</v>
@@ -9397,7 +9415,7 @@
         <v>0</v>
       </c>
       <c r="P130" s="2" t="n">
-        <v>46177</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="131">
@@ -9452,10 +9470,10 @@
         </is>
       </c>
       <c r="K131" s="2" t="n">
-        <v>46099</v>
+        <v>46102</v>
       </c>
       <c r="L131" s="2" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="M131" t="n">
         <v>127073.33</v>
@@ -9520,10 +9538,10 @@
         </is>
       </c>
       <c r="K132" s="2" t="n">
-        <v>46134</v>
+        <v>46137</v>
       </c>
       <c r="L132" s="2" t="n">
-        <v>46164</v>
+        <v>46167</v>
       </c>
       <c r="M132" t="n">
         <v>68707.3</v>
@@ -9588,7 +9606,7 @@
         </is>
       </c>
       <c r="K133" s="2" t="n">
-        <v>46219</v>
+        <v>46222</v>
       </c>
       <c r="L133" t="inlineStr"/>
       <c r="M133" t="n">

</xml_diff>